<commit_message>
Ajout de fonctionnalités dans plusieurs écrans
</commit_message>
<xml_diff>
--- a/Importation/Rencontres/Nationales_Ph_1_2026-2027.xlsx
+++ b/Importation/Rencontres/Nationales_Ph_1_2026-2027.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\wamp64\www\NIJAC\Importation\Rencontres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129E47CB-EACC-4E58-B018-94F2B9C7D5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8A17DC-DAB9-4A60-8565-42C36DDDC9A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="465" windowWidth="24210" windowHeight="15135" xr2:uid="{9E0913CB-4233-48FB-8E12-6DEFEB4AC469}"/>
+    <workbookView xWindow="2565" yWindow="105" windowWidth="24210" windowHeight="15135" activeTab="1" xr2:uid="{9E0913CB-4233-48FB-8E12-6DEFEB4AC469}"/>
   </bookViews>
   <sheets>
     <sheet name="Page 1" sheetId="1" r:id="rId1"/>
@@ -1094,7 +1094,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1128,6 +1128,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="13"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1258,7 +1264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1327,6 +1333,24 @@
     <xf numFmtId="1" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1336,6 +1360,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1345,37 +1393,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1390,109 +1426,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1894,26 +1903,26 @@
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:18" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="32"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:18" ht="13.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="32"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
       <c r="D10" s="35"/>
       <c r="E10" s="35"/>
       <c r="F10" s="35"/>
@@ -1925,40 +1934,40 @@
       <c r="A11" s="4">
         <v>1</v>
       </c>
-      <c r="B11" s="79">
+      <c r="B11" s="25">
         <v>46277</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="32"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:18" ht="2.4500000000000002" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="30">
+      <c r="A12" s="26">
         <v>2</v>
       </c>
-      <c r="B12" s="80">
+      <c r="B12" s="28">
         <v>46291</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="32"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:18" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="31"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
       <c r="D13" s="33"/>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -1975,9 +1984,9 @@
       <c r="Q13" s="33"/>
     </row>
     <row r="14" spans="1:18" ht="1.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="31"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
+      <c r="A14" s="27"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="35"/>
       <c r="E14" s="35"/>
       <c r="F14" s="35"/>
@@ -1986,26 +1995,26 @@
       <c r="I14" s="2"/>
     </row>
     <row r="15" spans="1:18" ht="2.4500000000000002" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="30">
+      <c r="A15" s="26">
         <v>3</v>
       </c>
-      <c r="B15" s="80">
+      <c r="B15" s="28">
         <v>46305</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="26"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="32"/>
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="1:18" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="31"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
       <c r="D16" s="33"/>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
@@ -2020,9 +2029,9 @@
       <c r="P16" s="33"/>
     </row>
     <row r="17" spans="1:16" ht="1.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="31"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
       <c r="D17" s="35"/>
       <c r="E17" s="35"/>
       <c r="F17" s="35"/>
@@ -2031,26 +2040,26 @@
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="1:16" ht="2.4500000000000002" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="30">
+      <c r="A18" s="26">
         <v>4</v>
       </c>
-      <c r="B18" s="80">
+      <c r="B18" s="28">
         <v>46340</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="32"/>
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="31"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
       <c r="D19" s="33"/>
       <c r="E19" s="33"/>
       <c r="F19" s="33"/>
@@ -2065,9 +2074,9 @@
       <c r="P19" s="33"/>
     </row>
     <row r="20" spans="1:16" ht="1.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="31"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
+      <c r="A20" s="27"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
       <c r="D20" s="35"/>
       <c r="E20" s="35"/>
       <c r="F20" s="35"/>
@@ -2076,26 +2085,26 @@
       <c r="I20" s="2"/>
     </row>
     <row r="21" spans="1:16" ht="2.4500000000000002" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="30">
+      <c r="A21" s="26">
         <v>5</v>
       </c>
-      <c r="B21" s="80">
+      <c r="B21" s="28">
         <v>46354</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="26"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="32"/>
       <c r="I21" s="2"/>
     </row>
     <row r="22" spans="1:16" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="31"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
       <c r="D22" s="33"/>
       <c r="E22" s="33"/>
       <c r="F22" s="33"/>
@@ -2108,9 +2117,9 @@
       <c r="O22" s="33"/>
     </row>
     <row r="23" spans="1:16" ht="1.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="31"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="32"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
       <c r="D23" s="35"/>
       <c r="E23" s="35"/>
       <c r="F23" s="35"/>
@@ -2122,34 +2131,34 @@
       <c r="A24" s="4">
         <v>6</v>
       </c>
-      <c r="B24" s="79">
+      <c r="B24" s="25">
         <v>46368</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="26"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="32"/>
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>7</v>
       </c>
-      <c r="B25" s="78">
+      <c r="B25" s="24">
         <v>46031</v>
       </c>
-      <c r="C25" s="27" t="s">
+      <c r="C25" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="29"/>
+      <c r="D25" s="42"/>
+      <c r="E25" s="42"/>
+      <c r="F25" s="42"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="43"/>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:16" ht="97.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -2169,6 +2178,16 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:H20"/>
+    <mergeCell ref="M19:P19"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="C21:H23"/>
+    <mergeCell ref="N22:O22"/>
     <mergeCell ref="A15:A17"/>
     <mergeCell ref="B15:B17"/>
     <mergeCell ref="C15:H17"/>
@@ -2185,16 +2204,6 @@
     <mergeCell ref="B12:B14"/>
     <mergeCell ref="C12:H14"/>
     <mergeCell ref="L13:Q13"/>
-    <mergeCell ref="M19:P19"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="C21:H23"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:H20"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2232,7 +2241,7 @@
       <c r="F1" s="6">
         <v>1</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="H1" s="50" t="s">
         <v>18</v>
       </c>
       <c r="I1" s="33"/>
@@ -2246,27 +2255,27 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:12" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="46"/>
+      <c r="B3" s="45"/>
       <c r="C3" s="2"/>
       <c r="H3" s="2"/>
-      <c r="I3" s="45" t="s">
+      <c r="I3" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="49"/>
-      <c r="K3" s="46"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="45"/>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
+      <c r="A4" s="46"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="47"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="48"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="47"/>
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2281,10 +2290,10 @@
       <c r="I5" s="9">
         <v>1</v>
       </c>
-      <c r="J5" s="41" t="s">
+      <c r="J5" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="42"/>
+      <c r="K5" s="52"/>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2299,10 +2308,10 @@
       <c r="I6" s="9">
         <v>2</v>
       </c>
-      <c r="J6" s="41" t="s">
+      <c r="J6" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="42"/>
+      <c r="K6" s="52"/>
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2317,10 +2326,10 @@
       <c r="I7" s="9">
         <v>3</v>
       </c>
-      <c r="J7" s="41" t="s">
+      <c r="J7" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="K7" s="42"/>
+      <c r="K7" s="52"/>
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2335,17 +2344,17 @@
       <c r="I8" s="9">
         <v>4</v>
       </c>
-      <c r="J8" s="41" t="s">
+      <c r="J8" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="K8" s="42"/>
+      <c r="K8" s="52"/>
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="81" t="s">
         <v>33</v>
       </c>
       <c r="C9" s="2"/>
@@ -2353,10 +2362,10 @@
       <c r="I9" s="9">
         <v>5</v>
       </c>
-      <c r="J9" s="41" t="s">
+      <c r="J9" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="K9" s="42"/>
+      <c r="K9" s="52"/>
       <c r="L9" s="2"/>
     </row>
     <row r="10" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2371,10 +2380,10 @@
       <c r="I10" s="9">
         <v>6</v>
       </c>
-      <c r="J10" s="41" t="s">
+      <c r="J10" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="K10" s="42"/>
+      <c r="K10" s="52"/>
       <c r="L10" s="2"/>
     </row>
     <row r="11" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2389,10 +2398,10 @@
       <c r="I11" s="9">
         <v>7</v>
       </c>
-      <c r="J11" s="41" t="s">
+      <c r="J11" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="42"/>
+      <c r="K11" s="52"/>
       <c r="L11" s="2"/>
     </row>
     <row r="12" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2407,10 +2416,10 @@
       <c r="I12" s="7">
         <v>8</v>
       </c>
-      <c r="J12" s="43" t="s">
+      <c r="J12" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="K12" s="44"/>
+      <c r="K12" s="54"/>
       <c r="L12" s="2"/>
     </row>
     <row r="13" spans="1:12" ht="27.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -2421,27 +2430,27 @@
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:12" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="45" t="s">
+      <c r="A14" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="46"/>
+      <c r="B14" s="45"/>
       <c r="C14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="45" t="s">
+      <c r="I14" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="J14" s="49"/>
-      <c r="K14" s="46"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="45"/>
       <c r="L14" s="2"/>
     </row>
     <row r="15" spans="1:12" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="47"/>
-      <c r="B15" s="48"/>
+      <c r="A15" s="46"/>
+      <c r="B15" s="47"/>
       <c r="C15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="47"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="48"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="47"/>
       <c r="L15" s="2"/>
     </row>
     <row r="16" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2456,10 +2465,10 @@
       <c r="I16" s="9">
         <v>1</v>
       </c>
-      <c r="J16" s="41" t="s">
+      <c r="J16" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="K16" s="42"/>
+      <c r="K16" s="52"/>
       <c r="L16" s="2"/>
     </row>
     <row r="17" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2474,10 +2483,10 @@
       <c r="I17" s="9">
         <v>2</v>
       </c>
-      <c r="J17" s="41" t="s">
+      <c r="J17" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="K17" s="42"/>
+      <c r="K17" s="52"/>
       <c r="L17" s="2"/>
     </row>
     <row r="18" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2492,10 +2501,10 @@
       <c r="I18" s="9">
         <v>3</v>
       </c>
-      <c r="J18" s="41" t="s">
+      <c r="J18" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="K18" s="42"/>
+      <c r="K18" s="52"/>
       <c r="L18" s="2"/>
     </row>
     <row r="19" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2510,10 +2519,10 @@
       <c r="I19" s="9">
         <v>4</v>
       </c>
-      <c r="J19" s="41" t="s">
+      <c r="J19" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="K19" s="42"/>
+      <c r="K19" s="52"/>
       <c r="L19" s="2"/>
     </row>
     <row r="20" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2528,10 +2537,10 @@
       <c r="I20" s="9">
         <v>5</v>
       </c>
-      <c r="J20" s="41" t="s">
+      <c r="J20" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="K20" s="42"/>
+      <c r="K20" s="52"/>
       <c r="L20" s="2"/>
     </row>
     <row r="21" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2546,10 +2555,10 @@
       <c r="I21" s="9">
         <v>6</v>
       </c>
-      <c r="J21" s="41" t="s">
+      <c r="J21" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="K21" s="42"/>
+      <c r="K21" s="52"/>
       <c r="L21" s="2"/>
     </row>
     <row r="22" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2564,10 +2573,10 @@
       <c r="I22" s="9">
         <v>7</v>
       </c>
-      <c r="J22" s="41" t="s">
+      <c r="J22" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="K22" s="42"/>
+      <c r="K22" s="52"/>
       <c r="L22" s="2"/>
     </row>
     <row r="23" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2582,10 +2591,10 @@
       <c r="I23" s="7">
         <v>8</v>
       </c>
-      <c r="J23" s="43" t="s">
+      <c r="J23" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="K23" s="44"/>
+      <c r="K23" s="54"/>
       <c r="L23" s="2"/>
     </row>
     <row r="24" spans="1:12" ht="88.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -2602,6 +2611,14 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
     <mergeCell ref="A14:B15"/>
     <mergeCell ref="I14:K15"/>
     <mergeCell ref="H1:J1"/>
@@ -2615,14 +2632,6 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="J11:K11"/>
     <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2653,7 +2662,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.850000000000001" customHeight="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="E1" s="60" t="s">
+      <c r="E1" s="55" t="s">
         <v>55</v>
       </c>
       <c r="F1" s="33"/>
@@ -2674,35 +2683,35 @@
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="53" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="53" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="I3" s="55"/>
-      <c r="J3" s="54"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="60"/>
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="57"/>
-      <c r="B4" s="58"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="59"/>
+      <c r="A4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="61"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2715,19 +2724,19 @@
       <c r="C5" s="14">
         <v>1</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
       <c r="H5" s="14">
         <v>1</v>
       </c>
-      <c r="I5" s="41" t="s">
+      <c r="I5" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="J5" s="42"/>
+      <c r="J5" s="52"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2740,19 +2749,19 @@
       <c r="C6" s="14">
         <v>2</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
       <c r="H6" s="14">
         <v>2</v>
       </c>
-      <c r="I6" s="41" t="s">
+      <c r="I6" s="51" t="s">
         <v>61</v>
       </c>
-      <c r="J6" s="42"/>
+      <c r="J6" s="52"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2765,19 +2774,19 @@
       <c r="C7" s="14">
         <v>3</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
       <c r="H7" s="14">
         <v>3</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="J7" s="42"/>
+      <c r="J7" s="52"/>
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2790,19 +2799,19 @@
       <c r="C8" s="14">
         <v>4</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="51" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
       <c r="H8" s="14">
         <v>4</v>
       </c>
-      <c r="I8" s="41" t="s">
+      <c r="I8" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="J8" s="42"/>
+      <c r="J8" s="52"/>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2815,19 +2824,19 @@
       <c r="C9" s="14">
         <v>5</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
       <c r="H9" s="14">
         <v>5</v>
       </c>
-      <c r="I9" s="41" t="s">
+      <c r="I9" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="42"/>
+      <c r="J9" s="52"/>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2840,19 +2849,19 @@
       <c r="C10" s="14">
         <v>6</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
       <c r="H10" s="14">
         <v>6</v>
       </c>
-      <c r="I10" s="41" t="s">
+      <c r="I10" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="42"/>
+      <c r="J10" s="52"/>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2865,19 +2874,19 @@
       <c r="C11" s="14">
         <v>7</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="56"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
       <c r="H11" s="14">
         <v>7</v>
       </c>
-      <c r="I11" s="41" t="s">
+      <c r="I11" s="51" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="42"/>
+      <c r="J11" s="52"/>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2890,19 +2899,19 @@
       <c r="C12" s="13">
         <v>8</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
       <c r="H12" s="13">
         <v>8</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="44"/>
+      <c r="J12" s="54"/>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2918,35 +2927,35 @@
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="53" t="s">
+      <c r="B14" s="57"/>
+      <c r="C14" s="56" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="53" t="s">
+      <c r="D14" s="57"/>
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="I14" s="55"/>
-      <c r="J14" s="54"/>
+      <c r="I14" s="57"/>
+      <c r="J14" s="60"/>
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="57"/>
-      <c r="B15" s="58"/>
-      <c r="C15" s="57"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="58"/>
-      <c r="J15" s="59"/>
+      <c r="A15" s="58"/>
+      <c r="B15" s="59"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="59"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="59"/>
+      <c r="J15" s="61"/>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2959,19 +2968,19 @@
       <c r="C16" s="14">
         <v>1</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="51" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
+      <c r="G16" s="62"/>
       <c r="H16" s="14">
         <v>1</v>
       </c>
-      <c r="I16" s="41" t="s">
+      <c r="I16" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="J16" s="42"/>
+      <c r="J16" s="52"/>
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -2984,19 +2993,19 @@
       <c r="C17" s="14">
         <v>2</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
       <c r="H17" s="14">
         <v>2</v>
       </c>
-      <c r="I17" s="41" t="s">
+      <c r="I17" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="J17" s="42"/>
+      <c r="J17" s="52"/>
       <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3009,19 +3018,19 @@
       <c r="C18" s="14">
         <v>3</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
+      <c r="G18" s="62"/>
       <c r="H18" s="14">
         <v>3</v>
       </c>
-      <c r="I18" s="41" t="s">
+      <c r="I18" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="J18" s="42"/>
+      <c r="J18" s="52"/>
       <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3034,19 +3043,19 @@
       <c r="C19" s="14">
         <v>4</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>93</v>
       </c>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
       <c r="H19" s="14">
         <v>4</v>
       </c>
-      <c r="I19" s="41" t="s">
+      <c r="I19" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="J19" s="42"/>
+      <c r="J19" s="52"/>
       <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3059,19 +3068,19 @@
       <c r="C20" s="14">
         <v>5</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="62"/>
       <c r="H20" s="14">
         <v>5</v>
       </c>
-      <c r="I20" s="41" t="s">
+      <c r="I20" s="51" t="s">
         <v>97</v>
       </c>
-      <c r="J20" s="42"/>
+      <c r="J20" s="52"/>
       <c r="K20" s="2"/>
     </row>
     <row r="21" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3084,19 +3093,19 @@
       <c r="C21" s="14">
         <v>6</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="51" t="s">
         <v>99</v>
       </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="62"/>
       <c r="H21" s="14">
         <v>6</v>
       </c>
-      <c r="I21" s="41" t="s">
+      <c r="I21" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="J21" s="42"/>
+      <c r="J21" s="52"/>
       <c r="K21" s="2"/>
     </row>
     <row r="22" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3109,19 +3118,19 @@
       <c r="C22" s="14">
         <v>7</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="51" t="s">
         <v>102</v>
       </c>
-      <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="62"/>
       <c r="H22" s="14">
         <v>7</v>
       </c>
-      <c r="I22" s="41" t="s">
+      <c r="I22" s="51" t="s">
         <v>103</v>
       </c>
-      <c r="J22" s="42"/>
+      <c r="J22" s="52"/>
       <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3134,19 +3143,19 @@
       <c r="C23" s="13">
         <v>8</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="63"/>
       <c r="H23" s="13">
         <v>8</v>
       </c>
-      <c r="I23" s="43" t="s">
+      <c r="I23" s="53" t="s">
         <v>106</v>
       </c>
-      <c r="J23" s="44"/>
+      <c r="J23" s="54"/>
       <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3169,17 +3178,17 @@
       <c r="J25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="20.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="53" t="s">
+      <c r="A26" s="56" t="s">
         <v>116</v>
       </c>
-      <c r="B26" s="54"/>
+      <c r="B26" s="60"/>
       <c r="C26" s="2"/>
       <c r="G26" s="2"/>
-      <c r="H26" s="53" t="s">
+      <c r="H26" s="56" t="s">
         <v>107</v>
       </c>
-      <c r="I26" s="55"/>
-      <c r="J26" s="54"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="60"/>
       <c r="K26" s="2"/>
     </row>
     <row r="27" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3194,10 +3203,10 @@
       <c r="H27" s="14">
         <v>1</v>
       </c>
-      <c r="I27" s="41" t="s">
+      <c r="I27" s="51" t="s">
         <v>108</v>
       </c>
-      <c r="J27" s="42"/>
+      <c r="J27" s="52"/>
       <c r="K27" s="2"/>
     </row>
     <row r="28" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3212,10 +3221,10 @@
       <c r="H28" s="14">
         <v>2</v>
       </c>
-      <c r="I28" s="41" t="s">
+      <c r="I28" s="51" t="s">
         <v>109</v>
       </c>
-      <c r="J28" s="42"/>
+      <c r="J28" s="52"/>
       <c r="K28" s="2"/>
     </row>
     <row r="29" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3230,10 +3239,10 @@
       <c r="H29" s="14">
         <v>3</v>
       </c>
-      <c r="I29" s="41" t="s">
+      <c r="I29" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="J29" s="42"/>
+      <c r="J29" s="52"/>
       <c r="K29" s="2"/>
     </row>
     <row r="30" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3248,10 +3257,10 @@
       <c r="H30" s="14">
         <v>4</v>
       </c>
-      <c r="I30" s="41" t="s">
+      <c r="I30" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="J30" s="42"/>
+      <c r="J30" s="52"/>
       <c r="K30" s="2"/>
     </row>
     <row r="31" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3266,10 +3275,10 @@
       <c r="H31" s="14">
         <v>5</v>
       </c>
-      <c r="I31" s="41" t="s">
+      <c r="I31" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="J31" s="42"/>
+      <c r="J31" s="52"/>
       <c r="K31" s="2"/>
     </row>
     <row r="32" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3284,10 +3293,10 @@
       <c r="H32" s="14">
         <v>6</v>
       </c>
-      <c r="I32" s="41" t="s">
+      <c r="I32" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="J32" s="42"/>
+      <c r="J32" s="52"/>
       <c r="K32" s="2"/>
     </row>
     <row r="33" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3302,10 +3311,10 @@
       <c r="H33" s="14">
         <v>7</v>
       </c>
-      <c r="I33" s="41" t="s">
+      <c r="I33" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="J33" s="42"/>
+      <c r="J33" s="52"/>
       <c r="K33" s="2"/>
     </row>
     <row r="34" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3320,10 +3329,10 @@
       <c r="H34" s="13">
         <v>8</v>
       </c>
-      <c r="I34" s="43" t="s">
+      <c r="I34" s="53" t="s">
         <v>115</v>
       </c>
-      <c r="J34" s="44"/>
+      <c r="J34" s="54"/>
       <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:11" ht="34.700000000000003" customHeight="1" x14ac:dyDescent="0.2">
@@ -3340,18 +3349,33 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:G4"/>
-    <mergeCell ref="H3:J4"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="A14:B15"/>
+    <mergeCell ref="C14:G15"/>
+    <mergeCell ref="H14:J15"/>
+    <mergeCell ref="D17:G17"/>
+    <mergeCell ref="I17:J17"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="D9:G9"/>
@@ -3362,33 +3386,18 @@
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="D12:G12"/>
     <mergeCell ref="I12:J12"/>
-    <mergeCell ref="A14:B15"/>
-    <mergeCell ref="C14:G15"/>
-    <mergeCell ref="H14:J15"/>
-    <mergeCell ref="D17:G17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:G4"/>
+    <mergeCell ref="H3:J4"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3427,7 +3436,7 @@
       <c r="G1" s="6">
         <v>3</v>
       </c>
-      <c r="I1" s="51" t="s">
+      <c r="I1" s="50" t="s">
         <v>18</v>
       </c>
       <c r="J1" s="33"/>
@@ -3448,39 +3457,39 @@
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="62"/>
-      <c r="C3" s="61" t="s">
+      <c r="B3" s="65"/>
+      <c r="C3" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="61" t="s">
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="64" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="68"/>
       <c r="M3" s="2"/>
     </row>
     <row r="4" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="64"/>
-      <c r="B4" s="65"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="65"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="65"/>
-      <c r="L4" s="66"/>
+      <c r="A4" s="66"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="66"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="69"/>
       <c r="M4" s="2"/>
     </row>
     <row r="5" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3493,21 +3502,21 @@
       <c r="C5" s="16">
         <v>1</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="56"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
       <c r="J5" s="16">
         <v>1</v>
       </c>
-      <c r="K5" s="41" t="s">
+      <c r="K5" s="51" t="s">
         <v>127</v>
       </c>
-      <c r="L5" s="42"/>
+      <c r="L5" s="52"/>
       <c r="M5" s="2"/>
     </row>
     <row r="6" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3520,21 +3529,21 @@
       <c r="C6" s="16">
         <v>2</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>129</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
       <c r="J6" s="16">
         <v>2</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K6" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="L6" s="42"/>
+      <c r="L6" s="52"/>
       <c r="M6" s="2"/>
     </row>
     <row r="7" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3547,21 +3556,21 @@
       <c r="C7" s="16">
         <v>3</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="51" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="56"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
       <c r="J7" s="16">
         <v>3</v>
       </c>
-      <c r="K7" s="41" t="s">
+      <c r="K7" s="51" t="s">
         <v>133</v>
       </c>
-      <c r="L7" s="42"/>
+      <c r="L7" s="52"/>
       <c r="M7" s="2"/>
     </row>
     <row r="8" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3574,21 +3583,21 @@
       <c r="C8" s="16">
         <v>4</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="51" t="s">
         <v>135</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="56"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
       <c r="J8" s="16">
         <v>4</v>
       </c>
-      <c r="K8" s="41" t="s">
+      <c r="K8" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="L8" s="42"/>
+      <c r="L8" s="52"/>
       <c r="M8" s="2"/>
     </row>
     <row r="9" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3601,21 +3610,21 @@
       <c r="C9" s="16">
         <v>5</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="56"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
       <c r="J9" s="16">
         <v>5</v>
       </c>
-      <c r="K9" s="41" t="s">
+      <c r="K9" s="51" t="s">
         <v>139</v>
       </c>
-      <c r="L9" s="42"/>
+      <c r="L9" s="52"/>
       <c r="M9" s="2"/>
     </row>
     <row r="10" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3628,21 +3637,21 @@
       <c r="C10" s="16">
         <v>6</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
       <c r="J10" s="16">
         <v>6</v>
       </c>
-      <c r="K10" s="41" t="s">
+      <c r="K10" s="51" t="s">
         <v>142</v>
       </c>
-      <c r="L10" s="42"/>
+      <c r="L10" s="52"/>
       <c r="M10" s="2"/>
     </row>
     <row r="11" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3655,21 +3664,21 @@
       <c r="C11" s="16">
         <v>7</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="E11" s="56"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
       <c r="J11" s="16">
         <v>7</v>
       </c>
-      <c r="K11" s="41" t="s">
+      <c r="K11" s="51" t="s">
         <v>145</v>
       </c>
-      <c r="L11" s="42"/>
+      <c r="L11" s="52"/>
       <c r="M11" s="2"/>
     </row>
     <row r="12" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3682,21 +3691,21 @@
       <c r="C12" s="15">
         <v>8</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
-      <c r="H12" s="52"/>
-      <c r="I12" s="52"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
       <c r="J12" s="15">
         <v>8</v>
       </c>
-      <c r="K12" s="43" t="s">
+      <c r="K12" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="L12" s="44"/>
+      <c r="L12" s="54"/>
       <c r="M12" s="2"/>
     </row>
     <row r="13" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3714,39 +3723,39 @@
       <c r="L13" s="2"/>
     </row>
     <row r="14" spans="1:13" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="62"/>
-      <c r="C14" s="61" t="s">
+      <c r="B14" s="65"/>
+      <c r="C14" s="64" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
-      <c r="G14" s="62"/>
-      <c r="H14" s="62"/>
-      <c r="I14" s="62"/>
-      <c r="J14" s="61" t="s">
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="64" t="s">
         <v>82</v>
       </c>
-      <c r="K14" s="62"/>
-      <c r="L14" s="63"/>
+      <c r="K14" s="65"/>
+      <c r="L14" s="68"/>
       <c r="M14" s="2"/>
     </row>
     <row r="15" spans="1:13" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="64"/>
-      <c r="B15" s="65"/>
-      <c r="C15" s="64"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
-      <c r="I15" s="65"/>
-      <c r="J15" s="64"/>
-      <c r="K15" s="65"/>
-      <c r="L15" s="66"/>
+      <c r="A15" s="66"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="66"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
+      <c r="I15" s="67"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="67"/>
+      <c r="L15" s="69"/>
       <c r="M15" s="2"/>
     </row>
     <row r="16" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3759,21 +3768,21 @@
       <c r="C16" s="16">
         <v>1</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="56"/>
-      <c r="I16" s="56"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
+      <c r="G16" s="62"/>
+      <c r="H16" s="62"/>
+      <c r="I16" s="62"/>
       <c r="J16" s="16">
         <v>1</v>
       </c>
-      <c r="K16" s="41" t="s">
+      <c r="K16" s="51" t="s">
         <v>151</v>
       </c>
-      <c r="L16" s="42"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="2"/>
     </row>
     <row r="17" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3786,21 +3795,21 @@
       <c r="C17" s="16">
         <v>2</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="56"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+      <c r="I17" s="62"/>
       <c r="J17" s="16">
         <v>2</v>
       </c>
-      <c r="K17" s="41" t="s">
+      <c r="K17" s="51" t="s">
         <v>154</v>
       </c>
-      <c r="L17" s="42"/>
+      <c r="L17" s="52"/>
       <c r="M17" s="2"/>
     </row>
     <row r="18" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3813,21 +3822,21 @@
       <c r="C18" s="16">
         <v>3</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="51" t="s">
         <v>156</v>
       </c>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="56"/>
-      <c r="I18" s="56"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
+      <c r="G18" s="62"/>
+      <c r="H18" s="62"/>
+      <c r="I18" s="62"/>
       <c r="J18" s="16">
         <v>3</v>
       </c>
-      <c r="K18" s="41" t="s">
+      <c r="K18" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="L18" s="42"/>
+      <c r="L18" s="52"/>
       <c r="M18" s="2"/>
     </row>
     <row r="19" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3840,21 +3849,21 @@
       <c r="C19" s="16">
         <v>4</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>159</v>
       </c>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+      <c r="H19" s="62"/>
+      <c r="I19" s="62"/>
       <c r="J19" s="16">
         <v>4</v>
       </c>
-      <c r="K19" s="41" t="s">
+      <c r="K19" s="51" t="s">
         <v>160</v>
       </c>
-      <c r="L19" s="42"/>
+      <c r="L19" s="52"/>
       <c r="M19" s="2"/>
     </row>
     <row r="20" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3867,21 +3876,21 @@
       <c r="C20" s="16">
         <v>5</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="51" t="s">
         <v>162</v>
       </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
-      <c r="H20" s="56"/>
-      <c r="I20" s="56"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="62"/>
+      <c r="H20" s="62"/>
+      <c r="I20" s="62"/>
       <c r="J20" s="16">
         <v>5</v>
       </c>
-      <c r="K20" s="41" t="s">
+      <c r="K20" s="51" t="s">
         <v>163</v>
       </c>
-      <c r="L20" s="42"/>
+      <c r="L20" s="52"/>
       <c r="M20" s="2"/>
     </row>
     <row r="21" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3894,21 +3903,21 @@
       <c r="C21" s="16">
         <v>6</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="51" t="s">
         <v>165</v>
       </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
-      <c r="H21" s="56"/>
-      <c r="I21" s="56"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="62"/>
+      <c r="H21" s="62"/>
+      <c r="I21" s="62"/>
       <c r="J21" s="16">
         <v>6</v>
       </c>
-      <c r="K21" s="41" t="s">
+      <c r="K21" s="51" t="s">
         <v>166</v>
       </c>
-      <c r="L21" s="42"/>
+      <c r="L21" s="52"/>
       <c r="M21" s="2"/>
     </row>
     <row r="22" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3921,21 +3930,21 @@
       <c r="C22" s="16">
         <v>7</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
-      <c r="I22" s="56"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="62"/>
+      <c r="H22" s="62"/>
+      <c r="I22" s="62"/>
       <c r="J22" s="16">
         <v>7</v>
       </c>
-      <c r="K22" s="41" t="s">
+      <c r="K22" s="51" t="s">
         <v>169</v>
       </c>
-      <c r="L22" s="42"/>
+      <c r="L22" s="52"/>
       <c r="M22" s="2"/>
     </row>
     <row r="23" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3948,21 +3957,21 @@
       <c r="C23" s="15">
         <v>8</v>
       </c>
-      <c r="D23" s="43" t="s">
+      <c r="D23" s="53" t="s">
         <v>171</v>
       </c>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
+      <c r="E23" s="63"/>
+      <c r="F23" s="63"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="63"/>
+      <c r="I23" s="63"/>
       <c r="J23" s="15">
         <v>8</v>
       </c>
-      <c r="K23" s="43" t="s">
+      <c r="K23" s="53" t="s">
         <v>172</v>
       </c>
-      <c r="L23" s="44"/>
+      <c r="L23" s="54"/>
       <c r="M23" s="2"/>
     </row>
     <row r="24" spans="1:13" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -3994,24 +4003,24 @@
       <c r="L25" s="2"/>
     </row>
     <row r="26" spans="1:13" ht="20.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="61" t="s">
+      <c r="A26" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="B26" s="62"/>
-      <c r="C26" s="61" t="s">
+      <c r="B26" s="65"/>
+      <c r="C26" s="64" t="s">
         <v>107</v>
       </c>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
-      <c r="G26" s="62"/>
-      <c r="H26" s="62"/>
-      <c r="I26" s="62"/>
-      <c r="J26" s="61" t="s">
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="65"/>
+      <c r="G26" s="65"/>
+      <c r="H26" s="65"/>
+      <c r="I26" s="65"/>
+      <c r="J26" s="64" t="s">
         <v>173</v>
       </c>
-      <c r="K26" s="62"/>
-      <c r="L26" s="63"/>
+      <c r="K26" s="65"/>
+      <c r="L26" s="68"/>
       <c r="M26" s="2"/>
     </row>
     <row r="27" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4024,21 +4033,21 @@
       <c r="C27" s="16">
         <v>1</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="51" t="s">
         <v>175</v>
       </c>
-      <c r="E27" s="56"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="56"/>
-      <c r="H27" s="56"/>
-      <c r="I27" s="56"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="62"/>
+      <c r="G27" s="62"/>
+      <c r="H27" s="62"/>
+      <c r="I27" s="62"/>
       <c r="J27" s="16">
         <v>1</v>
       </c>
-      <c r="K27" s="41" t="s">
+      <c r="K27" s="51" t="s">
         <v>176</v>
       </c>
-      <c r="L27" s="42"/>
+      <c r="L27" s="52"/>
       <c r="M27" s="2"/>
     </row>
     <row r="28" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4051,21 +4060,21 @@
       <c r="C28" s="16">
         <v>2</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="51" t="s">
         <v>178</v>
       </c>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="62"/>
+      <c r="G28" s="62"/>
+      <c r="H28" s="62"/>
+      <c r="I28" s="62"/>
       <c r="J28" s="16">
         <v>2</v>
       </c>
-      <c r="K28" s="41" t="s">
+      <c r="K28" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="L28" s="42"/>
+      <c r="L28" s="52"/>
       <c r="M28" s="2"/>
     </row>
     <row r="29" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4078,21 +4087,21 @@
       <c r="C29" s="16">
         <v>3</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="51" t="s">
         <v>181</v>
       </c>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
-      <c r="H29" s="56"/>
-      <c r="I29" s="56"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
+      <c r="I29" s="62"/>
       <c r="J29" s="16">
         <v>3</v>
       </c>
-      <c r="K29" s="41" t="s">
+      <c r="K29" s="51" t="s">
         <v>182</v>
       </c>
-      <c r="L29" s="42"/>
+      <c r="L29" s="52"/>
       <c r="M29" s="2"/>
     </row>
     <row r="30" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4105,21 +4114,21 @@
       <c r="C30" s="16">
         <v>4</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="51" t="s">
         <v>184</v>
       </c>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
-      <c r="H30" s="56"/>
-      <c r="I30" s="56"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="62"/>
+      <c r="H30" s="62"/>
+      <c r="I30" s="62"/>
       <c r="J30" s="16">
         <v>4</v>
       </c>
-      <c r="K30" s="41" t="s">
+      <c r="K30" s="51" t="s">
         <v>185</v>
       </c>
-      <c r="L30" s="42"/>
+      <c r="L30" s="52"/>
       <c r="M30" s="2"/>
     </row>
     <row r="31" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4132,21 +4141,21 @@
       <c r="C31" s="16">
         <v>5</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="51" t="s">
         <v>187</v>
       </c>
-      <c r="E31" s="56"/>
-      <c r="F31" s="56"/>
-      <c r="G31" s="56"/>
-      <c r="H31" s="56"/>
-      <c r="I31" s="56"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62"/>
+      <c r="H31" s="62"/>
+      <c r="I31" s="62"/>
       <c r="J31" s="16">
         <v>5</v>
       </c>
-      <c r="K31" s="41" t="s">
+      <c r="K31" s="51" t="s">
         <v>188</v>
       </c>
-      <c r="L31" s="42"/>
+      <c r="L31" s="52"/>
       <c r="M31" s="2"/>
     </row>
     <row r="32" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4159,21 +4168,21 @@
       <c r="C32" s="16">
         <v>6</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="51" t="s">
         <v>190</v>
       </c>
-      <c r="E32" s="56"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="56"/>
-      <c r="H32" s="56"/>
-      <c r="I32" s="56"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
+      <c r="H32" s="62"/>
+      <c r="I32" s="62"/>
       <c r="J32" s="16">
         <v>6</v>
       </c>
-      <c r="K32" s="41" t="s">
+      <c r="K32" s="51" t="s">
         <v>191</v>
       </c>
-      <c r="L32" s="42"/>
+      <c r="L32" s="52"/>
       <c r="M32" s="2"/>
     </row>
     <row r="33" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4186,21 +4195,21 @@
       <c r="C33" s="16">
         <v>7</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="51" t="s">
         <v>193</v>
       </c>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
-      <c r="H33" s="56"/>
-      <c r="I33" s="56"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
+      <c r="H33" s="62"/>
+      <c r="I33" s="62"/>
       <c r="J33" s="16">
         <v>7</v>
       </c>
-      <c r="K33" s="41" t="s">
+      <c r="K33" s="51" t="s">
         <v>194</v>
       </c>
-      <c r="L33" s="42"/>
+      <c r="L33" s="52"/>
       <c r="M33" s="2"/>
     </row>
     <row r="34" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4213,21 +4222,21 @@
       <c r="C34" s="15">
         <v>8</v>
       </c>
-      <c r="D34" s="43" t="s">
+      <c r="D34" s="53" t="s">
         <v>196</v>
       </c>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="52"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63"/>
       <c r="J34" s="15">
         <v>8</v>
       </c>
-      <c r="K34" s="43" t="s">
+      <c r="K34" s="53" t="s">
         <v>197</v>
       </c>
-      <c r="L34" s="44"/>
+      <c r="L34" s="54"/>
       <c r="M34" s="2"/>
     </row>
     <row r="35" spans="1:13" ht="49.7" customHeight="1" x14ac:dyDescent="0.2">
@@ -4251,33 +4260,23 @@
     </row>
   </sheetData>
   <mergeCells count="58">
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C3:I4"/>
-    <mergeCell ref="J3:L4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="D6:I6"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="D7:I7"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="D8:I8"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="D16:I16"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="D9:I9"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="D10:I10"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="D11:I11"/>
-    <mergeCell ref="K11:L11"/>
-    <mergeCell ref="D12:I12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="A14:B15"/>
-    <mergeCell ref="C14:I15"/>
-    <mergeCell ref="J14:L15"/>
-    <mergeCell ref="D17:I17"/>
-    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="D30:I30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="D34:I34"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="D31:I31"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="D32:I32"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="D33:I33"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C26:I26"/>
+    <mergeCell ref="J26:L26"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="K28:L28"/>
     <mergeCell ref="D18:I18"/>
     <mergeCell ref="K18:L18"/>
     <mergeCell ref="D19:I19"/>
@@ -4292,23 +4291,33 @@
     <mergeCell ref="K22:L22"/>
     <mergeCell ref="D23:I23"/>
     <mergeCell ref="K23:L23"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C26:I26"/>
-    <mergeCell ref="J26:L26"/>
-    <mergeCell ref="D28:I28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="D29:I29"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="D30:I30"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="D34:I34"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="D31:I31"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="D32:I32"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="D33:I33"/>
-    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="A14:B15"/>
+    <mergeCell ref="C14:I15"/>
+    <mergeCell ref="J14:L15"/>
+    <mergeCell ref="D17:I17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="D16:I16"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="D9:I9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="D10:I10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="D11:I11"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="D12:I12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="D8:I8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="A3:B4"/>
+    <mergeCell ref="C3:I4"/>
+    <mergeCell ref="J3:L4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="K5:L5"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4337,20 +4346,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="20.85" customHeight="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="64" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="61" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="64" t="s">
         <v>199</v>
       </c>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="61" t="s">
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="64" t="s">
         <v>200</v>
       </c>
-      <c r="H1" s="63"/>
+      <c r="H1" s="68"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4363,11 +4372,11 @@
       <c r="C2" s="16">
         <v>1</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="51" t="s">
         <v>202</v>
       </c>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
       <c r="G2" s="16">
         <v>1</v>
       </c>
@@ -4386,11 +4395,11 @@
       <c r="C3" s="16">
         <v>2</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="51" t="s">
         <v>205</v>
       </c>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
       <c r="G3" s="16">
         <v>2</v>
       </c>
@@ -4409,11 +4418,11 @@
       <c r="C4" s="16">
         <v>3</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="51" t="s">
         <v>208</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
       <c r="G4" s="16">
         <v>3</v>
       </c>
@@ -4432,11 +4441,11 @@
       <c r="C5" s="16">
         <v>4</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>211</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
       <c r="G5" s="16">
         <v>4</v>
       </c>
@@ -4455,11 +4464,11 @@
       <c r="C6" s="16">
         <v>5</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>214</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="16">
         <v>5</v>
       </c>
@@ -4478,11 +4487,11 @@
       <c r="C7" s="16">
         <v>6</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
       <c r="G7" s="16">
         <v>6</v>
       </c>
@@ -4501,11 +4510,11 @@
       <c r="C8" s="16">
         <v>7</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="16">
         <v>7</v>
       </c>
@@ -4524,11 +4533,11 @@
       <c r="C9" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="D9" s="43" t="s">
+      <c r="D9" s="53" t="s">
         <v>224</v>
       </c>
-      <c r="E9" s="52"/>
-      <c r="F9" s="52"/>
+      <c r="E9" s="63"/>
+      <c r="F9" s="63"/>
       <c r="G9" s="15">
         <v>8</v>
       </c>
@@ -4548,31 +4557,31 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:9" ht="0.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="64" t="s">
         <v>226</v>
       </c>
-      <c r="B11" s="62"/>
-      <c r="C11" s="61" t="s">
+      <c r="B11" s="65"/>
+      <c r="C11" s="64" t="s">
         <v>227</v>
       </c>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="61" t="s">
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="64" t="s">
         <v>228</v>
       </c>
-      <c r="H11" s="63"/>
+      <c r="H11" s="68"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:9" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="64"/>
-      <c r="B12" s="65"/>
-      <c r="C12" s="64"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="64"/>
-      <c r="H12" s="66"/>
+      <c r="A12" s="66"/>
+      <c r="B12" s="67"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="66"/>
+      <c r="H12" s="69"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4585,11 +4594,11 @@
       <c r="C13" s="16">
         <v>1</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="51" t="s">
         <v>230</v>
       </c>
-      <c r="E13" s="56"/>
-      <c r="F13" s="56"/>
+      <c r="E13" s="62"/>
+      <c r="F13" s="62"/>
       <c r="G13" s="16">
         <v>1</v>
       </c>
@@ -4608,11 +4617,11 @@
       <c r="C14" s="16">
         <v>2</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="51" t="s">
         <v>233</v>
       </c>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
       <c r="G14" s="16">
         <v>2</v>
       </c>
@@ -4631,11 +4640,11 @@
       <c r="C15" s="16">
         <v>3</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="51" t="s">
         <v>236</v>
       </c>
-      <c r="E15" s="56"/>
-      <c r="F15" s="56"/>
+      <c r="E15" s="62"/>
+      <c r="F15" s="62"/>
       <c r="G15" s="16">
         <v>3</v>
       </c>
@@ -4654,11 +4663,11 @@
       <c r="C16" s="16">
         <v>4</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="51" t="s">
         <v>239</v>
       </c>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
       <c r="G16" s="16">
         <v>4</v>
       </c>
@@ -4677,11 +4686,11 @@
       <c r="C17" s="16">
         <v>5</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="51" t="s">
         <v>242</v>
       </c>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
       <c r="G17" s="16">
         <v>5</v>
       </c>
@@ -4700,11 +4709,11 @@
       <c r="C18" s="16">
         <v>6</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="51" t="s">
         <v>245</v>
       </c>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
       <c r="G18" s="16">
         <v>6</v>
       </c>
@@ -4723,11 +4732,11 @@
       <c r="C19" s="16">
         <v>7</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>248</v>
       </c>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
       <c r="G19" s="16">
         <v>7</v>
       </c>
@@ -4746,11 +4755,11 @@
       <c r="C20" s="15">
         <v>8</v>
       </c>
-      <c r="D20" s="43" t="s">
+      <c r="D20" s="53" t="s">
         <v>251</v>
       </c>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
       <c r="G20" s="15">
         <v>8</v>
       </c>
@@ -4777,12 +4786,12 @@
     </row>
     <row r="23" spans="1:9" ht="20.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="2"/>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="64" t="s">
         <v>253</v>
       </c>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="63"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="68"/>
       <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4790,11 +4799,11 @@
       <c r="C24" s="16">
         <v>1</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="51" t="s">
         <v>254</v>
       </c>
-      <c r="E24" s="56"/>
-      <c r="F24" s="42"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="52"/>
       <c r="G24" s="2"/>
     </row>
     <row r="25" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4802,11 +4811,11 @@
       <c r="C25" s="16">
         <v>2</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="51" t="s">
         <v>255</v>
       </c>
-      <c r="E25" s="56"/>
-      <c r="F25" s="42"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="52"/>
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4814,11 +4823,11 @@
       <c r="C26" s="16">
         <v>3</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="51" t="s">
         <v>256</v>
       </c>
-      <c r="E26" s="56"/>
-      <c r="F26" s="42"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="52"/>
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4826,11 +4835,11 @@
       <c r="C27" s="16">
         <v>4</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="51" t="s">
         <v>257</v>
       </c>
-      <c r="E27" s="56"/>
-      <c r="F27" s="42"/>
+      <c r="E27" s="62"/>
+      <c r="F27" s="52"/>
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4838,11 +4847,11 @@
       <c r="C28" s="16">
         <v>5</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="51" t="s">
         <v>258</v>
       </c>
-      <c r="E28" s="56"/>
-      <c r="F28" s="42"/>
+      <c r="E28" s="62"/>
+      <c r="F28" s="52"/>
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4850,11 +4859,11 @@
       <c r="C29" s="16">
         <v>6</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="51" t="s">
         <v>259</v>
       </c>
-      <c r="E29" s="56"/>
-      <c r="F29" s="42"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="52"/>
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4862,11 +4871,11 @@
       <c r="C30" s="16">
         <v>7</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="51" t="s">
         <v>260</v>
       </c>
-      <c r="E30" s="56"/>
-      <c r="F30" s="42"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="52"/>
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4874,11 +4883,11 @@
       <c r="C31" s="15">
         <v>8</v>
       </c>
-      <c r="D31" s="43" t="s">
+      <c r="D31" s="53" t="s">
         <v>261</v>
       </c>
-      <c r="E31" s="52"/>
-      <c r="F31" s="44"/>
+      <c r="E31" s="63"/>
+      <c r="F31" s="54"/>
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:9" ht="50.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -4894,25 +4903,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A11:B12"/>
-    <mergeCell ref="C11:F12"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:F1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G11:H12"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
     <mergeCell ref="D31:F31"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="D19:F19"/>
@@ -4925,6 +4915,25 @@
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D29:F29"/>
     <mergeCell ref="D30:F30"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="A11:B12"/>
+    <mergeCell ref="C11:F12"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:F1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="G11:H12"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4955,7 +4964,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="17.850000000000001" customHeight="1" collapsed="1" x14ac:dyDescent="0.2">
-      <c r="E1" s="60" t="s">
+      <c r="E1" s="55" t="s">
         <v>262</v>
       </c>
       <c r="F1" s="33"/>
@@ -4977,22 +4986,22 @@
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="20.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="76"/>
-      <c r="C4" s="75" t="s">
+      <c r="B4" s="71"/>
+      <c r="C4" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="75" t="s">
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="76"/>
-      <c r="J4" s="77"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="72"/>
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5005,19 +5014,19 @@
       <c r="C5" s="20">
         <v>1</v>
       </c>
-      <c r="D5" s="41" t="s">
+      <c r="D5" s="51" t="s">
         <v>229</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="56"/>
-      <c r="G5" s="56"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
       <c r="H5" s="20">
         <v>1</v>
       </c>
-      <c r="I5" s="41" t="s">
+      <c r="I5" s="51" t="s">
         <v>264</v>
       </c>
-      <c r="J5" s="42"/>
+      <c r="J5" s="52"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5030,19 +5039,19 @@
       <c r="C6" s="20">
         <v>2</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="51" t="s">
         <v>265</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
       <c r="H6" s="20">
         <v>2</v>
       </c>
-      <c r="I6" s="41" t="s">
+      <c r="I6" s="51" t="s">
         <v>266</v>
       </c>
-      <c r="J6" s="42"/>
+      <c r="J6" s="52"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5055,19 +5064,19 @@
       <c r="C7" s="20">
         <v>3</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="51" t="s">
         <v>62</v>
       </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="56"/>
+      <c r="E7" s="62"/>
+      <c r="F7" s="62"/>
+      <c r="G7" s="62"/>
       <c r="H7" s="20">
         <v>3</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="51" t="s">
         <v>268</v>
       </c>
-      <c r="J7" s="42"/>
+      <c r="J7" s="52"/>
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5080,19 +5089,19 @@
       <c r="C8" s="20">
         <v>4</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="51" t="s">
         <v>270</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="56"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
       <c r="H8" s="20">
         <v>4</v>
       </c>
-      <c r="I8" s="41" t="s">
+      <c r="I8" s="51" t="s">
         <v>271</v>
       </c>
-      <c r="J8" s="42"/>
+      <c r="J8" s="52"/>
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5105,19 +5114,19 @@
       <c r="C9" s="20">
         <v>5</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="51" t="s">
         <v>273</v>
       </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="62"/>
+      <c r="G9" s="62"/>
       <c r="H9" s="20">
         <v>5</v>
       </c>
-      <c r="I9" s="41" t="s">
+      <c r="I9" s="51" t="s">
         <v>274</v>
       </c>
-      <c r="J9" s="42"/>
+      <c r="J9" s="52"/>
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5130,19 +5139,19 @@
       <c r="C10" s="20">
         <v>6</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="51" t="s">
         <v>276</v>
       </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
       <c r="H10" s="20">
         <v>6</v>
       </c>
-      <c r="I10" s="41" t="s">
+      <c r="I10" s="51" t="s">
         <v>277</v>
       </c>
-      <c r="J10" s="42"/>
+      <c r="J10" s="52"/>
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5155,19 +5164,19 @@
       <c r="C11" s="20">
         <v>7</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="51" t="s">
         <v>155</v>
       </c>
-      <c r="E11" s="56"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="62"/>
+      <c r="G11" s="62"/>
       <c r="H11" s="20">
         <v>7</v>
       </c>
-      <c r="I11" s="41" t="s">
+      <c r="I11" s="51" t="s">
         <v>278</v>
       </c>
-      <c r="J11" s="42"/>
+      <c r="J11" s="52"/>
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5180,19 +5189,19 @@
       <c r="C12" s="19">
         <v>8</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="53" t="s">
         <v>279</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="52"/>
-      <c r="G12" s="52"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
       <c r="H12" s="19">
         <v>8</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="53" t="s">
         <v>280</v>
       </c>
-      <c r="J12" s="44"/>
+      <c r="J12" s="54"/>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -5208,7 +5217,7 @@
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E14" s="60" t="s">
+      <c r="E14" s="55" t="s">
         <v>263</v>
       </c>
       <c r="F14" s="33"/>
@@ -5229,35 +5238,35 @@
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:11" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="69" t="s">
+      <c r="A16" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="70"/>
-      <c r="C16" s="69" t="s">
+      <c r="B16" s="74"/>
+      <c r="C16" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="69" t="s">
+      <c r="D16" s="74"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="I16" s="70"/>
-      <c r="J16" s="71"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="77"/>
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="20.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="72"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="72"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="73"/>
-      <c r="F17" s="73"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="72"/>
-      <c r="I17" s="73"/>
-      <c r="J17" s="74"/>
+      <c r="A17" s="75"/>
+      <c r="B17" s="76"/>
+      <c r="C17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="75"/>
+      <c r="I17" s="76"/>
+      <c r="J17" s="78"/>
       <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5270,19 +5279,19 @@
       <c r="C18" s="22">
         <v>1</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="51" t="s">
         <v>281</v>
       </c>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
+      <c r="G18" s="62"/>
       <c r="H18" s="22">
         <v>1</v>
       </c>
-      <c r="I18" s="41" t="s">
+      <c r="I18" s="51" t="s">
         <v>282</v>
       </c>
-      <c r="J18" s="42"/>
+      <c r="J18" s="52"/>
       <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5295,19 +5304,19 @@
       <c r="C19" s="22">
         <v>2</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
       <c r="H19" s="22">
         <v>2</v>
       </c>
-      <c r="I19" s="41" t="s">
+      <c r="I19" s="51" t="s">
         <v>283</v>
       </c>
-      <c r="J19" s="42"/>
+      <c r="J19" s="52"/>
       <c r="K19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5320,19 +5329,19 @@
       <c r="C20" s="22">
         <v>3</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="51" t="s">
         <v>285</v>
       </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="56"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="62"/>
       <c r="H20" s="22">
         <v>3</v>
       </c>
-      <c r="I20" s="41" t="s">
+      <c r="I20" s="51" t="s">
         <v>180</v>
       </c>
-      <c r="J20" s="42"/>
+      <c r="J20" s="52"/>
       <c r="K20" s="2"/>
     </row>
     <row r="21" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5345,19 +5354,19 @@
       <c r="C21" s="22">
         <v>4</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="51" t="s">
         <v>287</v>
       </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="56"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="62"/>
       <c r="H21" s="22">
         <v>4</v>
       </c>
-      <c r="I21" s="41" t="s">
+      <c r="I21" s="51" t="s">
         <v>288</v>
       </c>
-      <c r="J21" s="42"/>
+      <c r="J21" s="52"/>
       <c r="K21" s="2"/>
     </row>
     <row r="22" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5370,19 +5379,19 @@
       <c r="C22" s="22">
         <v>5</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="E22" s="56"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="56"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
+      <c r="G22" s="62"/>
       <c r="H22" s="22">
         <v>5</v>
       </c>
-      <c r="I22" s="41" t="s">
+      <c r="I22" s="51" t="s">
         <v>290</v>
       </c>
-      <c r="J22" s="42"/>
+      <c r="J22" s="52"/>
       <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5395,19 +5404,19 @@
       <c r="C23" s="22">
         <v>6</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="51" t="s">
         <v>292</v>
       </c>
-      <c r="E23" s="56"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="56"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
       <c r="H23" s="22">
         <v>6</v>
       </c>
-      <c r="I23" s="41" t="s">
+      <c r="I23" s="51" t="s">
         <v>293</v>
       </c>
-      <c r="J23" s="42"/>
+      <c r="J23" s="52"/>
       <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5420,19 +5429,19 @@
       <c r="C24" s="22">
         <v>7</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="56"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="56"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
+      <c r="G24" s="62"/>
       <c r="H24" s="22">
         <v>7</v>
       </c>
-      <c r="I24" s="41" t="s">
+      <c r="I24" s="51" t="s">
         <v>294</v>
       </c>
-      <c r="J24" s="42"/>
+      <c r="J24" s="52"/>
       <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5445,17 +5454,17 @@
       <c r="C25" s="21">
         <v>8</v>
       </c>
-      <c r="D25" s="67"/>
-      <c r="E25" s="68"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="68"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="80"/>
+      <c r="F25" s="80"/>
+      <c r="G25" s="80"/>
       <c r="H25" s="21">
         <v>8</v>
       </c>
-      <c r="I25" s="43" t="s">
+      <c r="I25" s="53" t="s">
         <v>295</v>
       </c>
-      <c r="J25" s="44"/>
+      <c r="J25" s="54"/>
       <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2">
@@ -5483,22 +5492,22 @@
       <c r="J27" s="2"/>
     </row>
     <row r="28" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="69" t="s">
+      <c r="A28" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="70"/>
-      <c r="C28" s="69" t="s">
+      <c r="B28" s="74"/>
+      <c r="C28" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="D28" s="70"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="70"/>
-      <c r="G28" s="70"/>
-      <c r="H28" s="69" t="s">
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="74"/>
+      <c r="H28" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="I28" s="70"/>
-      <c r="J28" s="71"/>
+      <c r="I28" s="74"/>
+      <c r="J28" s="77"/>
       <c r="K28" s="2"/>
     </row>
     <row r="29" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5511,19 +5520,19 @@
       <c r="C29" s="22">
         <v>1</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="51" t="s">
         <v>297</v>
       </c>
-      <c r="E29" s="56"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="56"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
       <c r="H29" s="22">
         <v>1</v>
       </c>
-      <c r="I29" s="41" t="s">
+      <c r="I29" s="51" t="s">
         <v>298</v>
       </c>
-      <c r="J29" s="42"/>
+      <c r="J29" s="52"/>
       <c r="K29" s="2"/>
     </row>
     <row r="30" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5536,19 +5545,19 @@
       <c r="C30" s="22">
         <v>2</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="51" t="s">
         <v>300</v>
       </c>
-      <c r="E30" s="56"/>
-      <c r="F30" s="56"/>
-      <c r="G30" s="56"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="62"/>
       <c r="H30" s="22">
         <v>2</v>
       </c>
-      <c r="I30" s="41" t="s">
+      <c r="I30" s="51" t="s">
         <v>301</v>
       </c>
-      <c r="J30" s="42"/>
+      <c r="J30" s="52"/>
       <c r="K30" s="2"/>
     </row>
     <row r="31" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5561,19 +5570,19 @@
       <c r="C31" s="22">
         <v>3</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="E31" s="56"/>
-      <c r="F31" s="56"/>
-      <c r="G31" s="56"/>
+      <c r="E31" s="62"/>
+      <c r="F31" s="62"/>
+      <c r="G31" s="62"/>
       <c r="H31" s="22">
         <v>3</v>
       </c>
-      <c r="I31" s="41" t="s">
+      <c r="I31" s="51" t="s">
         <v>63</v>
       </c>
-      <c r="J31" s="42"/>
+      <c r="J31" s="52"/>
       <c r="K31" s="2"/>
     </row>
     <row r="32" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5586,19 +5595,19 @@
       <c r="C32" s="23">
         <v>4</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="51" t="s">
         <v>303</v>
       </c>
-      <c r="E32" s="56"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="56"/>
+      <c r="E32" s="62"/>
+      <c r="F32" s="62"/>
+      <c r="G32" s="62"/>
       <c r="H32" s="22">
         <v>4</v>
       </c>
-      <c r="I32" s="41" t="s">
+      <c r="I32" s="51" t="s">
         <v>304</v>
       </c>
-      <c r="J32" s="42"/>
+      <c r="J32" s="52"/>
       <c r="K32" s="2"/>
     </row>
     <row r="33" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5611,19 +5620,19 @@
       <c r="C33" s="22">
         <v>5</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="51" t="s">
         <v>306</v>
       </c>
-      <c r="E33" s="56"/>
-      <c r="F33" s="56"/>
-      <c r="G33" s="56"/>
+      <c r="E33" s="62"/>
+      <c r="F33" s="62"/>
+      <c r="G33" s="62"/>
       <c r="H33" s="22">
         <v>5</v>
       </c>
-      <c r="I33" s="41" t="s">
+      <c r="I33" s="51" t="s">
         <v>307</v>
       </c>
-      <c r="J33" s="42"/>
+      <c r="J33" s="52"/>
       <c r="K33" s="2"/>
     </row>
     <row r="34" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5636,19 +5645,19 @@
       <c r="C34" s="22">
         <v>6</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="51" t="s">
         <v>309</v>
       </c>
-      <c r="E34" s="56"/>
-      <c r="F34" s="56"/>
-      <c r="G34" s="56"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
       <c r="H34" s="22">
         <v>6</v>
       </c>
-      <c r="I34" s="41" t="s">
+      <c r="I34" s="51" t="s">
         <v>310</v>
       </c>
-      <c r="J34" s="42"/>
+      <c r="J34" s="52"/>
       <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5661,19 +5670,19 @@
       <c r="C35" s="22">
         <v>7</v>
       </c>
-      <c r="D35" s="41" t="s">
+      <c r="D35" s="51" t="s">
         <v>312</v>
       </c>
-      <c r="E35" s="56"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
+      <c r="E35" s="62"/>
+      <c r="F35" s="62"/>
+      <c r="G35" s="62"/>
       <c r="H35" s="22">
         <v>7</v>
       </c>
-      <c r="I35" s="41" t="s">
+      <c r="I35" s="51" t="s">
         <v>313</v>
       </c>
-      <c r="J35" s="42"/>
+      <c r="J35" s="52"/>
       <c r="K35" s="2"/>
     </row>
     <row r="36" spans="1:11" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -5686,17 +5695,17 @@
       <c r="C36" s="21">
         <v>8</v>
       </c>
-      <c r="D36" s="67"/>
-      <c r="E36" s="68"/>
-      <c r="F36" s="68"/>
-      <c r="G36" s="68"/>
+      <c r="D36" s="79"/>
+      <c r="E36" s="80"/>
+      <c r="F36" s="80"/>
+      <c r="G36" s="80"/>
       <c r="H36" s="21">
         <v>8</v>
       </c>
-      <c r="I36" s="43" t="s">
+      <c r="I36" s="53" t="s">
         <v>314</v>
       </c>
-      <c r="J36" s="44"/>
+      <c r="J36" s="54"/>
       <c r="K36" s="2"/>
     </row>
     <row r="37" spans="1:11" ht="22.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -5718,55 +5727,6 @@
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="D5:G5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="A16:B17"/>
-    <mergeCell ref="C16:G17"/>
-    <mergeCell ref="H16:J17"/>
-    <mergeCell ref="D18:G18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="D19:G19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="D20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="D22:G22"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="I31:J31"/>
     <mergeCell ref="D35:G35"/>
     <mergeCell ref="I35:J35"/>
     <mergeCell ref="D36:G36"/>
@@ -5777,6 +5737,55 @@
     <mergeCell ref="I33:J33"/>
     <mergeCell ref="D34:G34"/>
     <mergeCell ref="I34:J34"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="D22:G22"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="D18:G18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="A16:B17"/>
+    <mergeCell ref="C16:G17"/>
+    <mergeCell ref="H16:J17"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <printOptions gridLines="1" gridLinesSet="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>